<commit_message>
data: publish 2026-09-24 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-24-182路.xlsx
+++ b/data/export/2026-09-24-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -632,32 +632,36 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:18</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>73分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -665,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:11</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -689,33 +693,37 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>73.0</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>2/12</t>
         </is>
       </c>
     </row>
@@ -743,32 +751,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>71分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -776,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:11</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,17 +812,17 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -820,13 +832,17 @@
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>71.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>1/12</t>
         </is>
       </c>
     </row>
@@ -887,7 +903,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:11</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -926,7 +942,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
@@ -937,7 +953,7 @@
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -998,7 +1014,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:11</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1048,7 +1064,7 @@
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1076,32 +1092,36 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>81分钟</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -1109,7 +1129,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:11</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1133,17 +1153,17 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr">
@@ -1153,13 +1173,17 @@
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB6" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>81.0</t>
+        </is>
+      </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>3/12</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1244,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:11</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1294,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1355,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:11</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1405,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1466,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:11</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1492,7 +1516,7 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1500,22 +1524,22 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>沪A67353D</t>
+          <t>沪A66513D</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>07:15</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1548,12 +1572,12 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1567,7 +1591,7 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
@@ -1603,7 +1627,566 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>73.0</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>2/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-09-24 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-24-182路.xlsx
+++ b/data/export/2026-09-24-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC55"/>
+  <dimension ref="A1:AC59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -827,22 +827,22 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>78.7</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>75.8</t>
+          <t>76.0</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>10:02</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1541,14 +1541,14 @@
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA9" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
           <t>82.0</t>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>12/14</t>
+          <t>13/14</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="AA10" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>75.7</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="AC10" s="2" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>12/14</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2141,17 +2141,17 @@
       </c>
       <c r="AA14" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
-          <t>82.3</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2493,22 +2493,22 @@
       </c>
       <c r="Z17" s="2" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AA17" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>78.7</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA19" s="2" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="AC19" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
-          <t>75.8</t>
+          <t>76.0</t>
         </is>
       </c>
       <c r="AC21" s="2" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>10:02</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -3207,14 +3207,14 @@
       </c>
       <c r="Z23" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA23" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
           <t>82.0</t>
@@ -3222,7 +3222,7 @@
       </c>
       <c r="AC23" s="2" t="inlineStr">
         <is>
-          <t>12/14</t>
+          <t>13/14</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="AA24" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
-          <t>75.7</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="AC24" s="2" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="AC25" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>12/14</t>
         </is>
       </c>
     </row>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3644,7 +3644,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA27" s="2" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3807,17 +3807,17 @@
       </c>
       <c r="AA28" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
-          <t>82.3</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC28" s="2" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -3882,7 +3882,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="AC29" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -4159,22 +4159,22 @@
       </c>
       <c r="Z31" s="2" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AA31" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
-          <t>78.7</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="AC31" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -4358,7 +4358,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="Z33" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA33" s="2" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="AC33" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
-          <t>75.8</t>
+          <t>76.0</t>
         </is>
       </c>
       <c r="AC35" s="2" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -4834,7 +4834,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -4878,12 +4878,12 @@
       </c>
       <c r="AA37" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
-          <t>75.7</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="AC37" s="2" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="AC38" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>12/14</t>
         </is>
       </c>
     </row>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="Z39" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA39" s="2" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -5235,17 +5235,17 @@
       </c>
       <c r="AA40" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
-          <t>82.3</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC40" s="2" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="AC42" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -5652,12 +5652,12 @@
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5759,24 +5759,24 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>71分钟</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr"/>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
-          <t>75.8</t>
+          <t>76.0</t>
         </is>
       </c>
       <c r="AC45" s="2" t="inlineStr">
@@ -5868,32 +5868,36 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>13:53</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>73分钟</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
           <t>06:41</t>
@@ -5901,7 +5905,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -5925,17 +5929,17 @@
       </c>
       <c r="W46" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X46" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y46" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z46" s="2" t="inlineStr">
@@ -5945,12 +5949,12 @@
       </c>
       <c r="AA46" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
-          <t>75.7</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="AC46" s="2" t="inlineStr">
@@ -6020,7 +6024,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -6102,32 +6106,36 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>77分钟</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
           <t>07:11</t>
@@ -6135,7 +6143,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -6159,17 +6167,17 @@
       </c>
       <c r="W48" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X48" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y48" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z48" s="2" t="inlineStr">
@@ -6179,17 +6187,17 @@
       </c>
       <c r="AA48" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
-          <t>82.3</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC48" s="2" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -6217,32 +6225,36 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>70分钟</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M49" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -6250,7 +6262,7 @@
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P49" s="2" t="inlineStr">
@@ -6274,37 +6286,37 @@
       </c>
       <c r="W49" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X49" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y49" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z49" s="2" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA49" s="2" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AA49" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
-          <t>78.7</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="AC49" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -6365,7 +6377,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -6419,7 +6431,7 @@
       </c>
       <c r="AC50" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -6480,7 +6492,7 @@
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P51" s="2" t="inlineStr">
@@ -6519,7 +6531,7 @@
       </c>
       <c r="Z51" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA51" s="2" t="inlineStr">
@@ -6534,7 +6546,7 @@
       </c>
       <c r="AC51" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -6595,7 +6607,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -6710,7 +6722,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -6825,7 +6837,7 @@
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
@@ -6940,7 +6952,7 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
@@ -6994,7 +7006,467 @@
       </c>
       <c r="AC55" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>12/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr"/>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr"/>
+      <c r="R56" s="2" t="inlineStr"/>
+      <c r="S56" s="2" t="inlineStr"/>
+      <c r="T56" s="2" t="inlineStr"/>
+      <c r="U56" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W56" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y56" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z56" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA56" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AB56" s="2" t="inlineStr">
+        <is>
+          <t>79.5</t>
+        </is>
+      </c>
+      <c r="AC56" s="2" t="inlineStr">
+        <is>
+          <t>8/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr"/>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="inlineStr"/>
+      <c r="R57" s="2" t="inlineStr"/>
+      <c r="S57" s="2" t="inlineStr"/>
+      <c r="T57" s="2" t="inlineStr"/>
+      <c r="U57" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y57" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z57" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA57" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AB57" s="2" t="inlineStr">
+        <is>
+          <t>76.5</t>
+        </is>
+      </c>
+      <c r="AC57" s="2" t="inlineStr">
+        <is>
+          <t>4/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr"/>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>沪A02126A</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>06:21</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr"/>
+      <c r="R58" s="2" t="inlineStr"/>
+      <c r="S58" s="2" t="inlineStr"/>
+      <c r="T58" s="2" t="inlineStr"/>
+      <c r="U58" s="2" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W58" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X58" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y58" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z58" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA58" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB58" s="2" t="inlineStr">
+        <is>
+          <t>82.0</t>
+        </is>
+      </c>
+      <c r="AC58" s="2" t="inlineStr">
+        <is>
+          <t>13/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr"/>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q59" s="2" t="inlineStr"/>
+      <c r="R59" s="2" t="inlineStr"/>
+      <c r="S59" s="2" t="inlineStr"/>
+      <c r="T59" s="2" t="inlineStr"/>
+      <c r="U59" s="2" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="V59" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W59" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X59" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y59" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z59" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA59" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB59" s="2" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
+      <c r="AC59" s="2" t="inlineStr">
+        <is>
+          <t>5/14</t>
         </is>
       </c>
     </row>

</xml_diff>